<commit_message>
data: actualiza operaciones.xlsx con nuevos datos
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/operaciones.xlsx
+++ b/operaciones.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD0E7901-79FA-4A07-BC95-6B301E9ADDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{291293E0-D776-408F-9700-73D630258304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="55">
   <si>
     <t>Fecha</t>
   </si>
@@ -1271,7 +1271,21 @@
       </c>
     </row>
     <row r="25" spans="1:21">
-      <c r="A25" s="1"/>
+      <c r="A25" s="1">
+        <v>45914</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25">
+        <v>5000</v>
+      </c>
       <c r="I25">
         <f>+I21+I20-I17</f>
         <v>12330</v>

</xml_diff>